<commit_message>
fix: label GPT.AX, GMG.AX and CHC.AX DCFs by their method, not the engine
All three run an AFFO / operating-profit stream at the cost of equity
through the Drivers route with net debt held at zero, but carried the
engine's default owner_fcf_dcf_component label, so sanity_check classed
them as owner-FCF. Relabelled in the Drivers file, rebuilt, price and
sanity blocks refreshed (affo / earnings_at_coe families), dashboards
re-embedded. Values unchanged.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/research/CHC.AX/Reports/CHC.AX_DCF_Model.xlsx
+++ b/research/CHC.AX/Reports/CHC.AX_DCF_Model.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="364" uniqueCount="167">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="368" uniqueCount="171">
   <si>
     <t xml:space="preserve">Ticker</t>
   </si>
@@ -64,7 +64,7 @@
     <t xml:space="preserve">Model</t>
   </si>
   <si>
-    <t xml:space="preserve">owner_fcf_dcf_component</t>
+    <t xml:space="preserve">REIT operating earnings capitalisation at cost of equity (engine route; funds management plus property trust)</t>
   </si>
   <si>
     <t xml:space="preserve">Currency (model)</t>
@@ -91,7 +91,7 @@
     <t xml:space="preserve">Built at</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-09-22T09:20:59Z</t>
+    <t xml:space="preserve">2026-09-22T20:11:28Z</t>
   </si>
   <si>
     <t xml:space="preserve">Drivers file</t>
@@ -224,6 +224,18 @@
   </si>
   <si>
     <t xml:space="preserve">TotalIncome</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FUM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OperatingEPS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OperatingEarnings</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PropertyFUM</t>
   </si>
   <si>
     <t xml:space="preserve">FY2016</t>
@@ -1014,7 +1026,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:AD12"/>
+  <dimension ref="A1:AH12"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1108,10 +1120,22 @@
       <c r="AD1" s="2" t="s">
         <v>64</v>
       </c>
+      <c r="AE1" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="AF1" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="AG1" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="AH1" s="2" t="s">
+        <v>68</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="B2" s="0" t="n">
         <v>145.055</v>
@@ -1155,10 +1179,16 @@
       <c r="AC2" s="0" t="n">
         <v>26.9</v>
       </c>
+      <c r="AF2" s="0" t="n">
+        <v>30.4</v>
+      </c>
+      <c r="AG2" s="0" t="n">
+        <v>124.7</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="B3" s="0" t="n">
         <v>213.393</v>
@@ -1208,10 +1238,16 @@
       <c r="AD3" s="0" t="n">
         <v>423.8</v>
       </c>
+      <c r="AF3" s="0" t="n">
+        <v>35.9</v>
+      </c>
+      <c r="AG3" s="0" t="n">
+        <v>151.2</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="B4" s="0" t="n">
         <v>246.2</v>
@@ -1261,10 +1297,22 @@
       <c r="AD4" s="0" t="n">
         <v>416.7</v>
       </c>
+      <c r="AE4" s="0" t="n">
+        <v>23.2</v>
+      </c>
+      <c r="AF4" s="0" t="n">
+        <v>37.7</v>
+      </c>
+      <c r="AG4" s="0" t="n">
+        <v>175.8</v>
+      </c>
+      <c r="AH4" s="0" t="n">
+        <v>23.2</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="B5" s="0" t="n">
         <v>378.5</v>
@@ -1317,10 +1365,22 @@
       <c r="AD5" s="0" t="n">
         <v>527.4</v>
       </c>
+      <c r="AE5" s="0" t="n">
+        <v>30.4</v>
+      </c>
+      <c r="AF5" s="0" t="n">
+        <v>47.4</v>
+      </c>
+      <c r="AG5" s="0" t="n">
+        <v>220.7</v>
+      </c>
+      <c r="AH5" s="0" t="n">
+        <v>30.4</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="B6" s="0" t="n">
         <v>553.8</v>
@@ -1373,10 +1433,22 @@
       <c r="AD6" s="0" t="n">
         <v>731.6</v>
       </c>
+      <c r="AE6" s="0" t="n">
+        <v>40.5</v>
+      </c>
+      <c r="AF6" s="0" t="n">
+        <v>69.3</v>
+      </c>
+      <c r="AG6" s="0" t="n">
+        <v>322.8</v>
+      </c>
+      <c r="AH6" s="0" t="n">
+        <v>40.5</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="B7" s="0" t="n">
         <v>668</v>
@@ -1426,10 +1498,22 @@
       <c r="AD7" s="0" t="n">
         <v>1011.4</v>
       </c>
+      <c r="AE7" s="0" t="n">
+        <v>52.3</v>
+      </c>
+      <c r="AF7" s="0" t="n">
+        <v>61</v>
+      </c>
+      <c r="AG7" s="0" t="n">
+        <v>284.3</v>
+      </c>
+      <c r="AH7" s="0" t="n">
+        <v>52.3</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="B8" s="0" t="n">
         <v>1098.3</v>
@@ -1479,10 +1563,22 @@
       <c r="AD8" s="0" t="n">
         <v>1666.7</v>
       </c>
+      <c r="AE8" s="0" t="n">
+        <v>79.9</v>
+      </c>
+      <c r="AF8" s="0" t="n">
+        <v>115.6</v>
+      </c>
+      <c r="AG8" s="0" t="n">
+        <v>542.8</v>
+      </c>
+      <c r="AH8" s="0" t="n">
+        <v>65.6</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="B9" s="0" t="n">
         <v>869.7</v>
@@ -1529,10 +1625,22 @@
       <c r="AC9" s="0" t="n">
         <v>42.5</v>
       </c>
+      <c r="AE9" s="0" t="n">
+        <v>87.4</v>
+      </c>
+      <c r="AF9" s="0" t="n">
+        <v>93.3</v>
+      </c>
+      <c r="AG9" s="0" t="n">
+        <v>441.2</v>
+      </c>
+      <c r="AH9" s="0" t="n">
+        <v>71.9</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="B10" s="0" t="n">
         <v>597.8</v>
@@ -1588,10 +1696,22 @@
       <c r="AD10" s="0" t="n">
         <v>597.8</v>
       </c>
+      <c r="AE10" s="0" t="n">
+        <v>80.9</v>
+      </c>
+      <c r="AF10" s="0" t="n">
+        <v>75.8</v>
+      </c>
+      <c r="AG10" s="0" t="n">
+        <v>358.7</v>
+      </c>
+      <c r="AH10" s="0" t="n">
+        <v>65.5</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="B11" s="0" t="n">
         <v>544.9</v>
@@ -1650,10 +1770,22 @@
       <c r="AD11" s="0" t="n">
         <v>687.8</v>
       </c>
+      <c r="AE11" s="0" t="n">
+        <v>84.3</v>
+      </c>
+      <c r="AF11" s="0" t="n">
+        <v>81.4</v>
+      </c>
+      <c r="AG11" s="0" t="n">
+        <v>385</v>
+      </c>
+      <c r="AH11" s="0" t="n">
+        <v>66.8</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="B12" s="0" t="n">
         <v>556.7</v>
@@ -1711,6 +1843,18 @@
       </c>
       <c r="AD12" s="0" t="n">
         <v>811.3</v>
+      </c>
+      <c r="AE12" s="0" t="n">
+        <v>94.3</v>
+      </c>
+      <c r="AF12" s="0" t="n">
+        <v>103.2</v>
+      </c>
+      <c r="AG12" s="0" t="n">
+        <v>488.1</v>
+      </c>
+      <c r="AH12" s="0" t="n">
+        <v>76</v>
       </c>
     </row>
   </sheetData>
@@ -1737,15 +1881,15 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="B2" s="3" t="n">
         <v>18.26</v>
@@ -1753,7 +1897,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="B3" s="3" t="n">
         <v>482.1</v>
@@ -1761,7 +1905,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="B4" s="3" t="n">
         <v>0</v>
@@ -1769,7 +1913,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="B5" s="3" t="n">
         <v>0</v>
@@ -1777,7 +1921,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="B6" s="3" t="n">
         <v>15</v>
@@ -1785,7 +1929,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="B7" s="3" t="n">
         <v>952.1</v>
@@ -1793,23 +1937,23 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="B10" s="3" t="n">
         <v>1</v>
@@ -1817,42 +1961,42 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="K12" s="2" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="L12" s="2" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="C13" s="3" t="n">
         <v>7</v>
@@ -1887,7 +2031,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="0" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C14" s="3" t="n">
         <v>60.5</v>
@@ -1922,7 +2066,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="0" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="C15" s="3" t="n">
         <v>0</v>
@@ -1957,7 +2101,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="0" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="C16" s="3" t="n">
         <v>0</v>
@@ -1992,7 +2136,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="0" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="C17" s="3" t="n">
         <v>0.9</v>
@@ -2027,7 +2171,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="0" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="C18" s="3" t="n">
         <v>27</v>
@@ -2062,7 +2206,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="0" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="C19" s="3" t="n">
         <v>15</v>
@@ -2097,7 +2241,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="0" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="B20" s="3" t="n">
         <v>10</v>
@@ -2105,7 +2249,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="0" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="B21" s="3" t="n">
         <v>2.5</v>
@@ -2113,7 +2257,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="0" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="B22" s="3" t="n">
         <v>15</v>
@@ -2121,7 +2265,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="0" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="B23" s="3" t="n">
         <v>0</v>
@@ -2129,7 +2273,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="0" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="B24" s="3" t="n">
         <v>0.25</v>
@@ -2137,42 +2281,42 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="I26" s="2" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="J26" s="2" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="K26" s="2" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="L26" s="2" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="0" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="C27" s="3" t="n">
         <v>10</v>
@@ -2207,7 +2351,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="0" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C28" s="3" t="n">
         <v>61</v>
@@ -2242,7 +2386,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="0" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="C29" s="3" t="n">
         <v>0</v>
@@ -2277,7 +2421,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="0" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="C30" s="3" t="n">
         <v>0</v>
@@ -2312,7 +2456,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="0" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="C31" s="3" t="n">
         <v>0.9</v>
@@ -2347,7 +2491,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="0" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="C32" s="3" t="n">
         <v>27</v>
@@ -2382,7 +2526,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="0" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="C33" s="3" t="n">
         <v>15</v>
@@ -2417,7 +2561,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="0" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="B34" s="3" t="n">
         <v>10</v>
@@ -2425,7 +2569,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="0" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="B35" s="3" t="n">
         <v>3</v>
@@ -2433,7 +2577,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="0" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="B36" s="3" t="n">
         <v>18</v>
@@ -2441,7 +2585,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="0" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="B37" s="3" t="n">
         <v>0</v>
@@ -2449,7 +2593,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="0" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="B38" s="3" t="n">
         <v>0.5</v>
@@ -2457,42 +2601,42 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="2" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="F40" s="2" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="G40" s="2" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="H40" s="2" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="I40" s="2" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="J40" s="2" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="K40" s="2" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="L40" s="2" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="0" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="C41" s="3" t="n">
         <v>13</v>
@@ -2527,7 +2671,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="0" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C42" s="3" t="n">
         <v>61.5</v>
@@ -2562,7 +2706,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="0" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="C43" s="3" t="n">
         <v>0</v>
@@ -2597,7 +2741,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="0" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="C44" s="3" t="n">
         <v>0</v>
@@ -2632,7 +2776,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="0" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="C45" s="3" t="n">
         <v>0.9</v>
@@ -2667,7 +2811,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="0" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="C46" s="3" t="n">
         <v>27</v>
@@ -2702,7 +2846,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="0" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="C47" s="3" t="n">
         <v>15</v>
@@ -2737,7 +2881,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="0" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="B48" s="3" t="n">
         <v>10</v>
@@ -2745,7 +2889,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="0" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="B49" s="3" t="n">
         <v>3.5</v>
@@ -2753,7 +2897,7 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="0" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="B50" s="3" t="n">
         <v>20</v>
@@ -2761,7 +2905,7 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="0" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="B51" s="3" t="n">
         <v>0</v>
@@ -2769,7 +2913,7 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="0" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="B52" s="3" t="n">
         <v>0.25</v>
@@ -2799,50 +2943,50 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="B4" s="0" t="n">
         <v>0</v>
@@ -2890,7 +3034,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="C5" s="4" t="n">
         <f aca="false">Assumptions!C13</f>
@@ -2983,7 +3127,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C7" s="4" t="n">
         <f aca="false">Assumptions!C14</f>
@@ -3073,7 +3217,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="C9" s="4" t="n">
         <f aca="false">Assumptions!C15</f>
@@ -3118,7 +3262,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="C10" s="0" t="n">
         <f aca="false">-C6*C9/100</f>
@@ -3163,7 +3307,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="C11" s="0" t="n">
         <f aca="false">C8+C10+C24</f>
@@ -3208,7 +3352,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="C12" s="4" t="n">
         <f aca="false">-C6*Assumptions!C17/100</f>
@@ -3253,7 +3397,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="C13" s="0" t="n">
         <f aca="false">C11+C12</f>
@@ -3298,7 +3442,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="0" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="C14" s="4" t="n">
         <f aca="false">Assumptions!C19</f>
@@ -3343,7 +3487,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="0" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="C15" s="0" t="n">
         <f aca="false">C13-MAX(0,C13)*C14/100</f>
@@ -3388,7 +3532,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="0" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="C16" s="0" t="n">
         <f aca="false">-C12</f>
@@ -3433,7 +3577,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="0" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="C17" s="4" t="n">
         <f aca="false">-C6*Assumptions!C18/100</f>
@@ -3478,7 +3622,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="0" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="C18" s="4" t="n">
         <f aca="false">(C6-B6)*Assumptions!$B$23/100</f>
@@ -3523,7 +3667,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="0" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="C19" s="0" t="n">
         <f aca="false">C15+C16+C17+C18</f>
@@ -3568,7 +3712,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="0" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="C20" s="0" t="n">
         <f aca="false">1/(1+$B$27/100)^C4</f>
@@ -3613,7 +3757,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="0" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="C21" s="0" t="n">
         <f aca="false">C19*C20</f>
@@ -3658,7 +3802,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="0" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="C23" s="4" t="n">
         <f aca="false">Assumptions!C16</f>
@@ -3703,7 +3847,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="0" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="C24" s="0" t="n">
         <f aca="false">-C6*C23/100</f>
@@ -3748,12 +3892,12 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="0" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="B27" s="4" t="n">
         <f aca="false">Assumptions!$B$20</f>
@@ -3762,7 +3906,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="0" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="B28" s="4" t="n">
         <f aca="false">Assumptions!$B$21</f>
@@ -3771,7 +3915,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="0" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="B29" s="4" t="n">
         <f aca="false">Assumptions!$B$22</f>
@@ -3780,7 +3924,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="0" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="B30" s="0" t="n">
         <f aca="false">SUM(C21:L21)</f>
@@ -3789,7 +3933,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="0" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="B31" s="0" t="n">
         <f aca="false">L19</f>
@@ -3798,7 +3942,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="0" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="B32" s="0" t="n">
         <f aca="false">IF(B27&gt;B28,B31*(1+B28/100)/((B27-B28)/100),B31*B29)</f>
@@ -3807,7 +3951,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="0" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="B33" s="0" t="n">
         <f aca="false">B31*B29</f>
@@ -3816,7 +3960,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="0" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="B34" s="0" t="n">
         <f aca="false">MAX(0,MIN(B32,B33))</f>
@@ -3825,7 +3969,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="0" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="B35" s="0" t="n">
         <f aca="false">B34/(1+B27/100)^L4</f>
@@ -3834,7 +3978,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="0" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="B36" s="0" t="n">
         <f aca="false">B30+B35</f>
@@ -3843,7 +3987,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="0" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="B37" s="0" t="n">
         <f aca="false">B36+Assumptions!$B$5-Assumptions!$B$4</f>
@@ -3852,7 +3996,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="0" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="B38" s="0" t="n">
         <f aca="false">B37/Assumptions!$B$3*Assumptions!$B$10</f>
@@ -3861,7 +4005,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="0" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="B39" s="4" t="n">
         <f aca="false">B38/Assumptions!$B$2-1</f>
@@ -3870,7 +4014,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="0" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="B41" s="0" t="n">
         <f aca="false">SUMPRODUCT(-C10:L10/(1+$B$27/100)^C4:L4)</f>
@@ -3879,7 +4023,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="0" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="B42" s="0" t="n">
         <f aca="false">IF(B27&gt;B28,-L10*(1+B28/100)/((B27-B28)/100),-L10*20)/(1+B27/100)^L4</f>
@@ -3888,7 +4032,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="0" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="B43" s="0" t="n">
         <f aca="false">(B37+B41+B42)/Assumptions!$B$3*Assumptions!$B$10</f>
@@ -3897,7 +4041,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="0" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="B45" s="4" t="n">
         <f aca="false">Assumptions!$B$6</f>
@@ -3906,7 +4050,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="0" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="B46" s="0" t="n">
         <f aca="false">MAX(0,MIN(IF(B45&gt;B28,B31*(1+B28/100)/((B45-B28)/100),B31*B29),B31*B29))</f>
@@ -3915,7 +4059,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="0" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="B47" s="0" t="n">
         <f aca="false">(SUMPRODUCT(C19:L19/(1+B45/100)^C4:L4)+B46/(1+B45/100)^L4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
@@ -3946,50 +4090,50 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="B4" s="0" t="n">
         <v>0</v>
@@ -4037,7 +4181,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="C5" s="4" t="n">
         <f aca="false">Assumptions!C27</f>
@@ -4130,7 +4274,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C7" s="4" t="n">
         <f aca="false">Assumptions!C28</f>
@@ -4220,7 +4364,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="C9" s="4" t="n">
         <f aca="false">Assumptions!C29</f>
@@ -4265,7 +4409,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="C10" s="0" t="n">
         <f aca="false">-C6*C9/100</f>
@@ -4310,7 +4454,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="C11" s="0" t="n">
         <f aca="false">C8+C10+C24</f>
@@ -4355,7 +4499,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="C12" s="4" t="n">
         <f aca="false">-C6*Assumptions!C31/100</f>
@@ -4400,7 +4544,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="C13" s="0" t="n">
         <f aca="false">C11+C12</f>
@@ -4445,7 +4589,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="0" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="C14" s="4" t="n">
         <f aca="false">Assumptions!C33</f>
@@ -4490,7 +4634,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="0" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="C15" s="0" t="n">
         <f aca="false">C13-MAX(0,C13)*C14/100</f>
@@ -4535,7 +4679,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="0" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="C16" s="0" t="n">
         <f aca="false">-C12</f>
@@ -4580,7 +4724,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="0" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="C17" s="4" t="n">
         <f aca="false">-C6*Assumptions!C32/100</f>
@@ -4625,7 +4769,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="0" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="C18" s="4" t="n">
         <f aca="false">(C6-B6)*Assumptions!$B$37/100</f>
@@ -4670,7 +4814,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="0" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="C19" s="0" t="n">
         <f aca="false">C15+C16+C17+C18</f>
@@ -4715,7 +4859,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="0" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="C20" s="0" t="n">
         <f aca="false">1/(1+$B$27/100)^C4</f>
@@ -4760,7 +4904,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="0" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="C21" s="0" t="n">
         <f aca="false">C19*C20</f>
@@ -4805,7 +4949,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="0" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="C23" s="4" t="n">
         <f aca="false">Assumptions!C30</f>
@@ -4850,7 +4994,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="0" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="C24" s="0" t="n">
         <f aca="false">-C6*C23/100</f>
@@ -4895,12 +5039,12 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="0" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="B27" s="4" t="n">
         <f aca="false">Assumptions!$B$34</f>
@@ -4909,7 +5053,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="0" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="B28" s="4" t="n">
         <f aca="false">Assumptions!$B$35</f>
@@ -4918,7 +5062,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="0" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="B29" s="4" t="n">
         <f aca="false">Assumptions!$B$36</f>
@@ -4927,7 +5071,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="0" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="B30" s="0" t="n">
         <f aca="false">SUM(C21:L21)</f>
@@ -4936,7 +5080,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="0" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="B31" s="0" t="n">
         <f aca="false">L19</f>
@@ -4945,7 +5089,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="0" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="B32" s="0" t="n">
         <f aca="false">IF(B27&gt;B28,B31*(1+B28/100)/((B27-B28)/100),B31*B29)</f>
@@ -4954,7 +5098,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="0" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="B33" s="0" t="n">
         <f aca="false">B31*B29</f>
@@ -4963,7 +5107,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="0" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="B34" s="0" t="n">
         <f aca="false">MAX(0,MIN(B32,B33))</f>
@@ -4972,7 +5116,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="0" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="B35" s="0" t="n">
         <f aca="false">B34/(1+B27/100)^L4</f>
@@ -4981,7 +5125,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="0" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="B36" s="0" t="n">
         <f aca="false">B30+B35</f>
@@ -4990,7 +5134,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="0" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="B37" s="0" t="n">
         <f aca="false">B36+Assumptions!$B$5-Assumptions!$B$4</f>
@@ -4999,7 +5143,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="0" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="B38" s="0" t="n">
         <f aca="false">B37/Assumptions!$B$3*Assumptions!$B$10</f>
@@ -5008,7 +5152,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="0" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="B39" s="4" t="n">
         <f aca="false">B38/Assumptions!$B$2-1</f>
@@ -5017,7 +5161,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="0" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="B41" s="0" t="n">
         <f aca="false">SUMPRODUCT(-C10:L10/(1+$B$27/100)^C4:L4)</f>
@@ -5026,7 +5170,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="0" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="B42" s="0" t="n">
         <f aca="false">IF(B27&gt;B28,-L10*(1+B28/100)/((B27-B28)/100),-L10*20)/(1+B27/100)^L4</f>
@@ -5035,7 +5179,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="0" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="B43" s="0" t="n">
         <f aca="false">(B37+B41+B42)/Assumptions!$B$3*Assumptions!$B$10</f>
@@ -5044,7 +5188,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="0" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="B45" s="4" t="n">
         <f aca="false">Assumptions!$B$6</f>
@@ -5053,7 +5197,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="0" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="B46" s="0" t="n">
         <f aca="false">MAX(0,MIN(IF(B45&gt;B28,B31*(1+B28/100)/((B45-B28)/100),B31*B29),B31*B29))</f>
@@ -5062,7 +5206,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="0" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="B47" s="0" t="n">
         <f aca="false">(SUMPRODUCT(C19:L19/(1+B45/100)^C4:L4)+B46/(1+B45/100)^L4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
@@ -5093,50 +5237,50 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="B4" s="0" t="n">
         <v>0</v>
@@ -5184,7 +5328,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="C5" s="4" t="n">
         <f aca="false">Assumptions!C41</f>
@@ -5277,7 +5421,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C7" s="4" t="n">
         <f aca="false">Assumptions!C42</f>
@@ -5367,7 +5511,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="C9" s="4" t="n">
         <f aca="false">Assumptions!C43</f>
@@ -5412,7 +5556,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="C10" s="0" t="n">
         <f aca="false">-C6*C9/100</f>
@@ -5457,7 +5601,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="C11" s="0" t="n">
         <f aca="false">C8+C10+C24</f>
@@ -5502,7 +5646,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="C12" s="4" t="n">
         <f aca="false">-C6*Assumptions!C45/100</f>
@@ -5547,7 +5691,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="C13" s="0" t="n">
         <f aca="false">C11+C12</f>
@@ -5592,7 +5736,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="0" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="C14" s="4" t="n">
         <f aca="false">Assumptions!C47</f>
@@ -5637,7 +5781,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="0" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="C15" s="0" t="n">
         <f aca="false">C13-MAX(0,C13)*C14/100</f>
@@ -5682,7 +5826,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="0" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="C16" s="0" t="n">
         <f aca="false">-C12</f>
@@ -5727,7 +5871,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="0" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="C17" s="4" t="n">
         <f aca="false">-C6*Assumptions!C46/100</f>
@@ -5772,7 +5916,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="0" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="C18" s="4" t="n">
         <f aca="false">(C6-B6)*Assumptions!$B$51/100</f>
@@ -5817,7 +5961,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="0" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="C19" s="0" t="n">
         <f aca="false">C15+C16+C17+C18</f>
@@ -5862,7 +6006,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="0" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="C20" s="0" t="n">
         <f aca="false">1/(1+$B$27/100)^C4</f>
@@ -5907,7 +6051,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="0" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="C21" s="0" t="n">
         <f aca="false">C19*C20</f>
@@ -5952,7 +6096,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="0" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="C23" s="4" t="n">
         <f aca="false">Assumptions!C44</f>
@@ -5997,7 +6141,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="0" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="C24" s="0" t="n">
         <f aca="false">-C6*C23/100</f>
@@ -6042,12 +6186,12 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="0" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="B27" s="4" t="n">
         <f aca="false">Assumptions!$B$48</f>
@@ -6056,7 +6200,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="0" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="B28" s="4" t="n">
         <f aca="false">Assumptions!$B$49</f>
@@ -6065,7 +6209,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="0" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="B29" s="4" t="n">
         <f aca="false">Assumptions!$B$50</f>
@@ -6074,7 +6218,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="0" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="B30" s="0" t="n">
         <f aca="false">SUM(C21:L21)</f>
@@ -6083,7 +6227,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="0" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="B31" s="0" t="n">
         <f aca="false">L19</f>
@@ -6092,7 +6236,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="0" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="B32" s="0" t="n">
         <f aca="false">IF(B27&gt;B28,B31*(1+B28/100)/((B27-B28)/100),B31*B29)</f>
@@ -6101,7 +6245,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="0" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="B33" s="0" t="n">
         <f aca="false">B31*B29</f>
@@ -6110,7 +6254,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="0" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="B34" s="0" t="n">
         <f aca="false">MAX(0,MIN(B32,B33))</f>
@@ -6119,7 +6263,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="0" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="B35" s="0" t="n">
         <f aca="false">B34/(1+B27/100)^L4</f>
@@ -6128,7 +6272,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="0" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="B36" s="0" t="n">
         <f aca="false">B30+B35</f>
@@ -6137,7 +6281,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="0" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="B37" s="0" t="n">
         <f aca="false">B36+Assumptions!$B$5-Assumptions!$B$4</f>
@@ -6146,7 +6290,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="0" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="B38" s="0" t="n">
         <f aca="false">B37/Assumptions!$B$3*Assumptions!$B$10</f>
@@ -6155,7 +6299,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="0" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="B39" s="4" t="n">
         <f aca="false">B38/Assumptions!$B$2-1</f>
@@ -6164,7 +6308,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="0" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="B41" s="0" t="n">
         <f aca="false">SUMPRODUCT(-C10:L10/(1+$B$27/100)^C4:L4)</f>
@@ -6173,7 +6317,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="0" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="B42" s="0" t="n">
         <f aca="false">IF(B27&gt;B28,-L10*(1+B28/100)/((B27-B28)/100),-L10*20)/(1+B27/100)^L4</f>
@@ -6182,7 +6326,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="0" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="B43" s="0" t="n">
         <f aca="false">(B37+B41+B42)/Assumptions!$B$3*Assumptions!$B$10</f>
@@ -6191,7 +6335,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="0" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="B45" s="4" t="n">
         <f aca="false">Assumptions!$B$6</f>
@@ -6200,7 +6344,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="0" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="B46" s="0" t="n">
         <f aca="false">MAX(0,MIN(IF(B45&gt;B28,B31*(1+B28/100)/((B45-B28)/100),B31*B29),B31*B29))</f>
@@ -6209,7 +6353,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="0" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="B47" s="0" t="n">
         <f aca="false">(SUMPRODUCT(C19:L19/(1+B45/100)^C4:L4)+B46/(1+B45/100)^L4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
@@ -6240,32 +6384,32 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="B4" s="4" t="n">
         <f aca="false">DCF_Bear!$B$38</f>
@@ -6290,7 +6434,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="B5" s="4" t="n">
         <f aca="false">DCF_Base!$B$38</f>
@@ -6315,7 +6459,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="B6" s="4" t="n">
         <f aca="false">DCF_Bull!$B$38</f>
@@ -6340,7 +6484,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="B8" s="0" t="n">
         <f aca="false">SUMPRODUCT(B4:B6,D4:D6)</f>
@@ -6349,7 +6493,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="B9" s="0" t="n">
         <f aca="false">SUMPRODUCT(E4:E6,D4:D6)</f>
@@ -6358,7 +6502,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="B10" s="0" t="n">
         <f aca="false">1-Assumptions!$B$2/B8</f>
@@ -6367,7 +6511,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="B11" s="0" t="str">
         <f aca="false">IF(ABS(B9-B8)&gt;0.01*ABS(B8),(Assumptions!$B$2-B8)/(B9-B8)*100,"n/a")</f>
@@ -6376,7 +6520,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="B12" s="0" t="n">
         <f aca="false">SUMPRODUCT(F4:F6,D4:D6)</f>
@@ -6385,15 +6529,15 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="C14" s="0" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="0" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="B15" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$C$15/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($C$15&gt;DCF_Base!$B$28,DCF_Base!$L$19*(1+DCF_Base!$B$28/100)/(($C$15-DCF_Base!$B$28)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$C$15/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
@@ -6405,7 +6549,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="0" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="B16" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$C$16/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($C$16&gt;DCF_Base!$B$28,DCF_Base!$L$19*(1+DCF_Base!$B$28/100)/(($C$16-DCF_Base!$B$28)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$C$16/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
@@ -6417,7 +6561,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="0" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="B17" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$C$17/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($C$17&gt;DCF_Base!$B$28,DCF_Base!$L$19*(1+DCF_Base!$B$28/100)/(($C$17-DCF_Base!$B$28)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$C$17/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
@@ -6429,7 +6573,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="0" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="B18" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$C$18/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($C$18&gt;DCF_Base!$B$28,DCF_Base!$L$19*(1+DCF_Base!$B$28/100)/(($C$18-DCF_Base!$B$28)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$C$18/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
@@ -6441,7 +6585,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="0" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="B19" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$C$19/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($C$19&gt;DCF_Base!$B$28,DCF_Base!$L$19*(1+DCF_Base!$B$28/100)/(($C$19-DCF_Base!$B$28)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$C$19/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
@@ -6453,7 +6597,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>